<commit_message>
Correcao qtd imoveis nas planilhas: IMMU, SEMASC E SEMJEL
</commit_message>
<xml_diff>
--- a/arquivos/SEMJEL/bemimovel_jan2026_semjel.xlsx
+++ b/arquivos/SEMJEL/bemimovel_jan2026_semjel.xlsx
@@ -19,7 +19,7 @@
     <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bens Imóveis'!$A$3:$Z$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bens Imóveis'!$A$3:$Z$23</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="201">
   <si>
     <t>ENDEREÇO</t>
   </si>
@@ -157,105 +157,69 @@
     <t>SECRETARIA</t>
   </si>
   <si>
-    <t>01101</t>
-  </si>
-  <si>
     <t>Câmara Municipal de Manaus</t>
   </si>
   <si>
     <t>CC</t>
   </si>
   <si>
-    <t>11101</t>
-  </si>
-  <si>
     <t>Casa Civil</t>
   </si>
   <si>
     <t>CC-ERB</t>
   </si>
   <si>
-    <t>11103</t>
-  </si>
-  <si>
     <t>GVP</t>
   </si>
   <si>
-    <t>12101</t>
-  </si>
-  <si>
     <t>Gabinete do Vice-Prefeito</t>
   </si>
   <si>
     <t>PGM</t>
   </si>
   <si>
-    <t>13101</t>
-  </si>
-  <si>
     <t>Procuradoria Geral do Municipio</t>
   </si>
   <si>
     <t>SEMAD</t>
   </si>
   <si>
-    <t>14101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Administração e Gestão</t>
   </si>
   <si>
     <t>CM</t>
   </si>
   <si>
-    <t>15101</t>
-  </si>
-  <si>
     <t>Casa Militar</t>
   </si>
   <si>
     <t>SEMEF</t>
   </si>
   <si>
-    <t>16101</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Secretaria Municipal de Finanças, Planejamento e Tecnologia da Informação</t>
   </si>
   <si>
     <t>SEMED</t>
   </si>
   <si>
-    <t>18101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Educação</t>
   </si>
   <si>
     <t>SEMCOM</t>
   </si>
   <si>
-    <t>19101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Comunicação</t>
   </si>
   <si>
     <t>SEMTEPI</t>
   </si>
   <si>
-    <t>21101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal do Trabalho, Empreendedorismo e Inovação</t>
   </si>
   <si>
     <t>CGM</t>
   </si>
   <si>
-    <t>22101</t>
-  </si>
-  <si>
     <t>Controladoria Geral do Municipio</t>
   </si>
   <si>
@@ -265,9 +229,6 @@
     <t>FMS</t>
   </si>
   <si>
-    <t>23701</t>
-  </si>
-  <si>
     <t>Fundo Municipal de Saúde</t>
   </si>
   <si>
@@ -277,33 +238,21 @@
     <t>SEMSEG</t>
   </si>
   <si>
-    <t>25101</t>
-  </si>
-  <si>
     <t>SEMJEL</t>
   </si>
   <si>
-    <t>26101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Juventude, Esporte e Lazer</t>
   </si>
   <si>
     <t>SEMINF</t>
   </si>
   <si>
-    <t>27101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Infraestrutura</t>
   </si>
   <si>
     <t>SEMMAS</t>
   </si>
   <si>
-    <t>28101</t>
-  </si>
-  <si>
     <t>Secretaria de Meio Ambiente e Sustentabilidade</t>
   </si>
   <si>
@@ -313,78 +262,51 @@
     <t>Secretaria Municipal da Mulher, Assistência Social e Cidadania</t>
   </si>
   <si>
-    <t>37101</t>
-  </si>
-  <si>
     <t>SEMULSP</t>
   </si>
   <si>
-    <t>38101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Limpeza Urbana</t>
   </si>
   <si>
     <t>SEMACC</t>
   </si>
   <si>
-    <t>41101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Agricultura, Abastecimento, Centro e Comércio Informal</t>
   </si>
   <si>
     <t>SEMHAF</t>
   </si>
   <si>
-    <t>44101</t>
-  </si>
-  <si>
     <t>Secretaria Municipal de Habitação e Assuntos Fundiários</t>
   </si>
   <si>
     <t>FDT</t>
   </si>
   <si>
-    <t>52301</t>
-  </si>
-  <si>
     <t>Fundação Doutor Thomas</t>
   </si>
   <si>
     <t>IMPLURB</t>
   </si>
   <si>
-    <t>56201</t>
-  </si>
-  <si>
     <t>Instituto Municipal de Planejamento Urbano</t>
   </si>
   <si>
     <t>IMMU</t>
   </si>
   <si>
-    <t>58201</t>
-  </si>
-  <si>
     <t>Instituto Municipal de Mobilidade Urbana</t>
   </si>
   <si>
     <t>MANAUSCULT</t>
   </si>
   <si>
-    <t>62301</t>
-  </si>
-  <si>
     <t>Fundação Municipal de Cultura, Turismo e Eventos</t>
   </si>
   <si>
     <t>MANAUSPREV</t>
   </si>
   <si>
-    <t>63201</t>
-  </si>
-  <si>
     <t>Manaus Previdência</t>
   </si>
   <si>
@@ -394,9 +316,6 @@
     <t>Agência Reguladora dos Serviços Públicos Delegados do Município de Manaus</t>
   </si>
   <si>
-    <t>70201</t>
-  </si>
-  <si>
     <t>Escritório de Representação em Brasília</t>
   </si>
   <si>
@@ -431,9 +350,6 @@
   </si>
   <si>
     <t>SEMSA</t>
-  </si>
-  <si>
-    <t>23000</t>
   </si>
   <si>
     <t>Secretaria Municipal de Saúde</t>
@@ -638,10 +554,88 @@
     <t>Rua 01, S/N - Armando Mendes - CEP 69.000-000</t>
   </si>
   <si>
-    <t>Rua Castro Alves, S/N - Aleixo - CEP 69.060-040</t>
-  </si>
-  <si>
-    <t>Parque Cidade da Criança</t>
+    <t>700201</t>
+  </si>
+  <si>
+    <t>110101</t>
+  </si>
+  <si>
+    <t>110103</t>
+  </si>
+  <si>
+    <t>220101</t>
+  </si>
+  <si>
+    <t>150101</t>
+  </si>
+  <si>
+    <t>010101</t>
+  </si>
+  <si>
+    <t>520301</t>
+  </si>
+  <si>
+    <t>230701</t>
+  </si>
+  <si>
+    <t>120101</t>
+  </si>
+  <si>
+    <t>580201</t>
+  </si>
+  <si>
+    <t>560201</t>
+  </si>
+  <si>
+    <t>620301</t>
+  </si>
+  <si>
+    <t>630201</t>
+  </si>
+  <si>
+    <t>130101</t>
+  </si>
+  <si>
+    <t>410101</t>
+  </si>
+  <si>
+    <t>140101</t>
+  </si>
+  <si>
+    <t>370101</t>
+  </si>
+  <si>
+    <t>190101</t>
+  </si>
+  <si>
+    <t>180101</t>
+  </si>
+  <si>
+    <t>160101</t>
+  </si>
+  <si>
+    <t>440101</t>
+  </si>
+  <si>
+    <t>270101</t>
+  </si>
+  <si>
+    <t>260101</t>
+  </si>
+  <si>
+    <t>280101</t>
+  </si>
+  <si>
+    <t>230101</t>
+  </si>
+  <si>
+    <t>250101</t>
+  </si>
+  <si>
+    <t>210101</t>
+  </si>
+  <si>
+    <t>380101</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="4" bestFit="1" customWidth="1"/>
@@ -1251,10 +1245,10 @@
     </row>
     <row r="2" spans="1:26" s="18" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -1266,81 +1260,81 @@
       <c r="J2" s="17"/>
       <c r="K2" s="14"/>
       <c r="L2" s="17" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
       <c r="M2" s="16" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="N2" s="15" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="O2" s="15" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="Q2" s="15" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="R2" s="15" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="S2" s="15" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="T2" s="15" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="U2" s="15" t="s">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="V2" s="15" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="W2" s="15" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="X2" s="15" t="s">
-        <v>160</v>
+        <v>132</v>
       </c>
       <c r="Y2" s="15" t="s">
-        <v>161</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:26" s="2" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>142</v>
+        <v>114</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>143</v>
+        <v>115</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>146</v>
+        <v>118</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="K3" s="11" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="L3" s="11" t="s">
         <v>3</v>
@@ -1355,7 +1349,7 @@
         <v>7</v>
       </c>
       <c r="P3" s="11" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="Q3" s="11" t="s">
         <v>0</v>
@@ -1367,7 +1361,7 @@
         <v>9</v>
       </c>
       <c r="T3" s="11" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="U3" s="11" t="s">
         <v>10</v>
@@ -1387,31 +1381,31 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B4" s="3" t="str">
         <f>VLOOKUP(A4,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F4" s="22"/>
       <c r="G4" s="22"/>
       <c r="H4" s="24"/>
       <c r="I4" s="24">
-        <f t="shared" ref="I4:I24" si="0">H4+L4</f>
+        <f t="shared" ref="I4:I22" si="0">H4+L4</f>
         <v>0</v>
       </c>
       <c r="J4" s="22"/>
       <c r="K4" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L4" s="24">
         <v>0</v>
@@ -1420,59 +1414,59 @@
         <v>505</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O4" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P4" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q4" s="23" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="R4" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S4" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T4" s="8" t="str">
         <f>VLOOKUP(A4,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U4" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V4" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W4" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X4" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y4" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B5" s="3" t="str">
         <f>VLOOKUP(A5,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F5" s="22"/>
       <c r="G5" s="22"/>
@@ -1483,7 +1477,7 @@
       </c>
       <c r="J5" s="22"/>
       <c r="K5" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L5" s="24">
         <v>0</v>
@@ -1492,59 +1486,59 @@
         <v>506</v>
       </c>
       <c r="N5" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O5" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P5" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q5" s="23" t="s">
-        <v>182</v>
+        <v>154</v>
       </c>
       <c r="R5" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S5" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T5" s="8" t="str">
         <f>VLOOKUP(A5,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U5" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V5" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W5" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X5" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y5" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B6" s="3" t="str">
         <f>VLOOKUP(A6,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>164</v>
+        <v>136</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F6" s="22"/>
       <c r="G6" s="22"/>
@@ -1555,7 +1549,7 @@
       </c>
       <c r="J6" s="22"/>
       <c r="K6" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L6" s="24">
         <v>0</v>
@@ -1564,59 +1558,59 @@
         <v>507</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q6" s="23" t="s">
-        <v>183</v>
+        <v>155</v>
       </c>
       <c r="R6" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S6" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T6" s="8" t="str">
         <f>VLOOKUP(A6,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U6" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V6" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W6" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X6" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y6" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B7" s="3" t="str">
         <f>VLOOKUP(A7,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>165</v>
+        <v>137</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F7" s="22"/>
       <c r="G7" s="22"/>
@@ -1627,7 +1621,7 @@
       </c>
       <c r="J7" s="22"/>
       <c r="K7" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L7" s="24">
         <v>0</v>
@@ -1636,59 +1630,59 @@
         <v>508</v>
       </c>
       <c r="N7" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O7" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q7" s="23" t="s">
-        <v>184</v>
+        <v>156</v>
       </c>
       <c r="R7" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S7" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T7" s="8" t="str">
         <f>VLOOKUP(A7,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U7" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V7" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W7" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X7" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y7" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B8" s="3" t="str">
         <f>VLOOKUP(A8,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F8" s="22"/>
       <c r="G8" s="22"/>
@@ -1699,7 +1693,7 @@
       </c>
       <c r="J8" s="22"/>
       <c r="K8" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L8" s="24">
         <v>0</v>
@@ -1708,59 +1702,59 @@
         <v>509</v>
       </c>
       <c r="N8" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O8" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P8" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q8" s="23" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
       <c r="R8" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S8" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T8" s="8" t="str">
         <f>VLOOKUP(A8,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U8" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V8" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W8" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X8" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y8" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B9" s="3" t="str">
         <f>VLOOKUP(A9,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>167</v>
+        <v>139</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F9" s="22"/>
       <c r="G9" s="22"/>
@@ -1771,7 +1765,7 @@
       </c>
       <c r="J9" s="22"/>
       <c r="K9" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L9" s="24">
         <v>0</v>
@@ -1780,59 +1774,59 @@
         <v>510</v>
       </c>
       <c r="N9" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O9" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P9" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q9" s="23" t="s">
-        <v>186</v>
+        <v>158</v>
       </c>
       <c r="R9" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S9" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T9" s="8" t="str">
         <f>VLOOKUP(A9,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U9" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V9" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W9" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X9" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y9" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B10" s="3" t="str">
         <f>VLOOKUP(A10,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F10" s="22"/>
       <c r="G10" s="22"/>
@@ -1843,7 +1837,7 @@
       </c>
       <c r="J10" s="22"/>
       <c r="K10" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L10" s="24">
         <v>0</v>
@@ -1852,59 +1846,59 @@
         <v>511</v>
       </c>
       <c r="N10" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O10" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P10" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q10" s="23" t="s">
-        <v>187</v>
+        <v>159</v>
       </c>
       <c r="R10" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S10" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T10" s="8" t="str">
         <f>VLOOKUP(A10,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U10" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V10" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W10" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X10" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y10" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B11" s="3" t="str">
         <f>VLOOKUP(A11,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="22"/>
@@ -1915,7 +1909,7 @@
       </c>
       <c r="J11" s="22"/>
       <c r="K11" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L11" s="24">
         <v>0</v>
@@ -1924,59 +1918,59 @@
         <v>512</v>
       </c>
       <c r="N11" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O11" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P11" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q11" s="23" t="s">
-        <v>188</v>
+        <v>160</v>
       </c>
       <c r="R11" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S11" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T11" s="8" t="str">
         <f>VLOOKUP(A11,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U11" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V11" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W11" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X11" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y11" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B12" s="3" t="str">
         <f>VLOOKUP(A12,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F12" s="22"/>
       <c r="G12" s="22"/>
@@ -1987,7 +1981,7 @@
       </c>
       <c r="J12" s="22"/>
       <c r="K12" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L12" s="24">
         <v>0</v>
@@ -1996,59 +1990,59 @@
         <v>513</v>
       </c>
       <c r="N12" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O12" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P12" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q12" s="23" t="s">
-        <v>189</v>
+        <v>161</v>
       </c>
       <c r="R12" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S12" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T12" s="8" t="str">
         <f>VLOOKUP(A12,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U12" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V12" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W12" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X12" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y12" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B13" s="3" t="str">
         <f>VLOOKUP(A13,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F13" s="22"/>
       <c r="G13" s="22"/>
@@ -2059,7 +2053,7 @@
       </c>
       <c r="J13" s="22"/>
       <c r="K13" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L13" s="24">
         <v>0</v>
@@ -2068,59 +2062,59 @@
         <v>514</v>
       </c>
       <c r="N13" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O13" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P13" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q13" s="23" t="s">
-        <v>190</v>
+        <v>162</v>
       </c>
       <c r="R13" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S13" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T13" s="8" t="str">
         <f>VLOOKUP(A13,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U13" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V13" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W13" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X13" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y13" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B14" s="3" t="str">
         <f>VLOOKUP(A14,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>172</v>
+        <v>144</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F14" s="22"/>
       <c r="G14" s="22"/>
@@ -2131,7 +2125,7 @@
       </c>
       <c r="J14" s="22"/>
       <c r="K14" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L14" s="24">
         <v>0</v>
@@ -2140,59 +2134,59 @@
         <v>515</v>
       </c>
       <c r="N14" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O14" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P14" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q14" s="23" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
       <c r="R14" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S14" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T14" s="8" t="str">
         <f>VLOOKUP(A14,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U14" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V14" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W14" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X14" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y14" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B15" s="3" t="str">
         <f>VLOOKUP(A15,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>173</v>
+        <v>145</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F15" s="22"/>
       <c r="G15" s="22"/>
@@ -2203,7 +2197,7 @@
       </c>
       <c r="J15" s="22"/>
       <c r="K15" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L15" s="24">
         <v>0</v>
@@ -2212,59 +2206,59 @@
         <v>516</v>
       </c>
       <c r="N15" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O15" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P15" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q15" s="23" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="R15" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S15" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T15" s="8" t="str">
         <f>VLOOKUP(A15,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U15" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V15" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W15" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X15" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y15" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B16" s="3" t="str">
         <f>VLOOKUP(A16,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>174</v>
+        <v>146</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F16" s="22"/>
       <c r="G16" s="22"/>
@@ -2275,7 +2269,7 @@
       </c>
       <c r="J16" s="22"/>
       <c r="K16" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L16" s="24">
         <v>0</v>
@@ -2284,59 +2278,59 @@
         <v>517</v>
       </c>
       <c r="N16" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O16" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P16" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q16" s="23" t="s">
-        <v>193</v>
+        <v>165</v>
       </c>
       <c r="R16" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S16" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T16" s="8" t="str">
         <f>VLOOKUP(A16,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U16" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V16" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W16" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X16" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y16" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B17" s="3" t="str">
         <f>VLOOKUP(A17,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F17" s="22"/>
       <c r="G17" s="22"/>
@@ -2347,7 +2341,7 @@
       </c>
       <c r="J17" s="22"/>
       <c r="K17" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L17" s="24">
         <v>0</v>
@@ -2356,59 +2350,59 @@
         <v>518</v>
       </c>
       <c r="N17" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O17" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P17" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q17" s="23" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="R17" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S17" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T17" s="8" t="str">
         <f>VLOOKUP(A17,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U17" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V17" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W17" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X17" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y17" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A18" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B18" s="3" t="str">
         <f>VLOOKUP(A18,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F18" s="22"/>
       <c r="G18" s="22"/>
@@ -2419,7 +2413,7 @@
       </c>
       <c r="J18" s="22"/>
       <c r="K18" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L18" s="24">
         <v>0</v>
@@ -2428,59 +2422,59 @@
         <v>519</v>
       </c>
       <c r="N18" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O18" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P18" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q18" s="23" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
       <c r="R18" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S18" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T18" s="8" t="str">
         <f>VLOOKUP(A18,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U18" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V18" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W18" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X18" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y18" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B19" s="3" t="str">
         <f>VLOOKUP(A19,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F19" s="22"/>
       <c r="G19" s="22"/>
@@ -2491,7 +2485,7 @@
       </c>
       <c r="J19" s="22"/>
       <c r="K19" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L19" s="24">
         <v>0</v>
@@ -2500,62 +2494,62 @@
         <v>520</v>
       </c>
       <c r="N19" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O19" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P19" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q19" s="23" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="R19" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S19" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T19" s="8" t="str">
         <f>VLOOKUP(A19,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U19" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V19" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W19" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X19" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y19" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B20" s="3" t="str">
         <f>VLOOKUP(A20,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="G20" s="22">
         <v>12635</v>
@@ -2569,7 +2563,7 @@
         <v>44431</v>
       </c>
       <c r="K20" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L20" s="24">
         <v>1476959.12</v>
@@ -2578,62 +2572,62 @@
         <v>521</v>
       </c>
       <c r="N20" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O20" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P20" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q20" s="23" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
       <c r="R20" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S20" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T20" s="8" t="str">
         <f>VLOOKUP(A20,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U20" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V20" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W20" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X20" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y20" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B21" s="3" t="str">
         <f>VLOOKUP(A21,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="G21" s="22">
         <v>27915</v>
@@ -2645,7 +2639,7 @@
       </c>
       <c r="J21" s="22"/>
       <c r="K21" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L21" s="24">
         <v>0</v>
@@ -2654,59 +2648,59 @@
         <v>522</v>
       </c>
       <c r="N21" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O21" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P21" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q21" s="23" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="R21" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S21" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T21" s="8" t="str">
         <f>VLOOKUP(A21,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U21" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V21" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W21" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X21" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y21" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A22" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B22" s="3" t="str">
         <f>VLOOKUP(A22,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F22" s="22"/>
       <c r="G22" s="22"/>
@@ -2717,7 +2711,7 @@
       </c>
       <c r="J22" s="22"/>
       <c r="K22" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L22" s="24">
         <v>0</v>
@@ -2726,59 +2720,59 @@
         <v>523</v>
       </c>
       <c r="N22" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O22" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P22" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q22" s="23" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
       <c r="R22" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S22" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T22" s="8" t="str">
         <f>VLOOKUP(A22,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U22" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V22" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W22" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X22" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y22" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23" s="22" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B23" s="3" t="str">
         <f>VLOOKUP(A23,Listas!A$3:C$30,3,0)</f>
         <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="F23" s="22"/>
       <c r="G23" s="22"/>
@@ -2789,7 +2783,7 @@
       </c>
       <c r="J23" s="22"/>
       <c r="K23" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="L23" s="24">
         <v>0</v>
@@ -2798,113 +2792,41 @@
         <v>524</v>
       </c>
       <c r="N23" s="25" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="O23" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="P23" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Q23" s="23" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
       <c r="R23" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="S23" s="22" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="T23" s="8" t="str">
         <f>VLOOKUP(A23,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
+        <v>260101</v>
       </c>
       <c r="U23" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="V23" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="W23" s="20" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="X23" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="Y23" s="19" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A24" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B24" s="3" t="str">
-        <f>VLOOKUP(A24,Listas!A$3:C$30,3,0)</f>
-        <v>Secretaria Municipal de Juventude, Esporte e Lazer</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>128</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="L24" s="24">
-        <v>0</v>
-      </c>
-      <c r="M24" s="21">
-        <v>525</v>
-      </c>
-      <c r="N24" s="25" t="s">
-        <v>138</v>
-      </c>
-      <c r="O24" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="P24" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q24" s="23" t="s">
-        <v>201</v>
-      </c>
-      <c r="R24" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="S24" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="T24" s="8" t="str">
-        <f>VLOOKUP(A24,Listas!A$3:C$30,2,0)</f>
-        <v>26101</v>
-      </c>
-      <c r="U24" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="V24" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="W24" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="X24" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="Y24" s="19" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2917,7 +2839,7 @@
           <x14:formula1>
             <xm:f>'N:\DPAT\_GESTÃO DE IMÓVEIS\1.INFORMAÇÕES IMÓVEIS\IMÓVEIS COM REGISTRO E SEM REGISTRO\[BEM IMÓVEL - SEMJEL_ajuste.xlsx]Listas'!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>A4:A24 S4:S24 P4:P24 D4:D24</xm:sqref>
+          <xm:sqref>A4:A23 S4:S23 P4:P23 D4:D23</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2941,7 +2863,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>40</v>
@@ -2961,13 +2883,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>118</v>
+        <v>92</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>119</v>
+        <v>93</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>18</v>
@@ -2984,13 +2906,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>17</v>
@@ -3007,13 +2929,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>47</v>
+        <v>175</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>19</v>
@@ -3030,16 +2952,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>73</v>
+        <v>176</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>24</v>
@@ -3053,13 +2975,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>58</v>
+        <v>177</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
@@ -3077,31 +2999,31 @@
         <v>39</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>42</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>104</v>
+        <v>179</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
@@ -3112,13 +3034,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>77</v>
+        <v>180</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
@@ -3129,13 +3051,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -3144,13 +3066,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>110</v>
+        <v>182</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -3159,13 +3081,13 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>107</v>
+        <v>183</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
@@ -3174,13 +3096,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>113</v>
+        <v>184</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -3189,13 +3111,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>116</v>
+        <v>185</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
@@ -3204,13 +3126,13 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>52</v>
+        <v>186</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
@@ -3219,13 +3141,13 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>98</v>
+        <v>187</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
@@ -3234,13 +3156,13 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>55</v>
+        <v>188</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
@@ -3249,13 +3171,13 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>93</v>
+        <v>189</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
@@ -3264,13 +3186,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>67</v>
+        <v>190</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
@@ -3279,13 +3201,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>64</v>
+        <v>191</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
@@ -3294,13 +3216,13 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>61</v>
+        <v>192</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
@@ -3309,13 +3231,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>101</v>
+        <v>193</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
@@ -3324,13 +3246,13 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>86</v>
+        <v>194</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
@@ -3339,13 +3261,13 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>83</v>
+        <v>195</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
@@ -3354,13 +3276,13 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>89</v>
+        <v>196</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -3369,13 +3291,13 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>133</v>
+        <v>197</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
@@ -3384,13 +3306,13 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>81</v>
+        <v>198</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
@@ -3399,13 +3321,13 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>70</v>
+        <v>199</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -3414,13 +3336,13 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>

</xml_diff>